<commit_message>
Add Ex3A to week-01
</commit_message>
<xml_diff>
--- a/week-01/Ex2B_data_roundup.xlsx
+++ b/week-01/Ex2B_data_roundup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sguer\Documents\DataAnalytics\week-01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE07B85F-9606-44B8-B0D7-60DE9FD48889}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F91C225-0DDC-4752-BE6B-DB6652E18A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{A12C3710-4084-4616-9F21-66122AF96B42}"/>
+    <workbookView xWindow="1222" yWindow="1305" windowWidth="16200" windowHeight="11813" xr2:uid="{A12C3710-4084-4616-9F21-66122AF96B42}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -368,6 +368,9 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DEF9BF44-0BE0-4E00-8A0A-CAD2BBEB7FC9}" name="Table1" displayName="Table1" ref="A1:G5" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5" headerRowCellStyle="Heading 4">
   <autoFilter ref="A1:G5" xr:uid="{DEF9BF44-0BE0-4E00-8A0A-CAD2BBEB7FC9}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G5">
+    <sortCondition ref="A1:A5"/>
+  </sortState>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{C9960577-0959-4650-AC69-BC15458F7638}" name="Name Of Data Source" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{E9882D06-C471-4FE2-B352-2641FBBFD9B0}" name="Type of Info" dataDxfId="3"/>
@@ -745,27 +748,27 @@
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
     </row>
-    <row r="2" spans="1:21" ht="180.4" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:21" ht="166.5" x14ac:dyDescent="0.45">
       <c r="A2" s="5" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>13</v>
+        <v>18</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>19</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
@@ -780,27 +783,27 @@
       <c r="R2" s="1"/>
       <c r="S2" s="1"/>
     </row>
-    <row r="3" spans="1:21" ht="166.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:21" ht="152.65" x14ac:dyDescent="0.45">
       <c r="A3" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="8" t="s">
-        <v>25</v>
+      <c r="C3" s="7" t="s">
+        <v>23</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="7" t="s">
         <v>19</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
@@ -815,27 +818,27 @@
       <c r="R3" s="1"/>
       <c r="S3" s="1"/>
     </row>
-    <row r="4" spans="1:21" ht="180.4" x14ac:dyDescent="0.45">
-      <c r="A4" s="5" t="s">
-        <v>7</v>
+    <row r="4" spans="1:21" ht="97.15" x14ac:dyDescent="0.45">
+      <c r="A4" s="6" t="s">
+        <v>9</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="7" t="s">
-        <v>23</v>
+      <c r="C4" s="8" t="s">
+        <v>26</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>19</v>
+      <c r="E4" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>27</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
@@ -850,27 +853,27 @@
       <c r="R4" s="1"/>
       <c r="S4" s="1"/>
     </row>
-    <row r="5" spans="1:21" ht="97.15" x14ac:dyDescent="0.45">
-      <c r="A5" s="6" t="s">
-        <v>9</v>
+    <row r="5" spans="1:21" ht="138.75" x14ac:dyDescent="0.45">
+      <c r="A5" s="5" t="s">
+        <v>6</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>27</v>
+      <c r="E5" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>13</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>

</xml_diff>